<commit_message>
Update the results to the corrected inputs and add the downscaling sensitivity
- City input table: the night-time light tile between 10°W and 0° and 40°N
  and 75°N, absent from the exported 2025 VIIRS monthly composites, is filled
  from the 2024 annual VIIRS Nighttime Lights composite (Supplementary Note 2).
- step_07 and step_05e read the 21-tier rating scale of _code/llm/tier_to_score.py,
  so A- ratings enter the vulnerability ratio and the vote fallback uses the
  correct tier values.
- Results of run v28_full5862_viirsfill_tierfix_20261021 replace those of
  v28_full5862_20260702_020421; the model ratings are unchanged.
- New _code/plotting_v28_full5862/downscaling_sensitivity.py and its tables
  (Supplementary Note 3 and Supplementary Table 4).
- Analysis tables, figure source data and analysis/mainline_diagnostics.py
  regenerated from the new run; the US county join keeps only identifiers and
  FEMA NRI scores.
</commit_message>
<xml_diff>
--- a/source_data/Extended_Data_Fig_1_source_data.xlsx
+++ b/source_data/Extended_Data_Fig_1_source_data.xlsx
@@ -462,7 +462,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>a, Mean GCIRI of cities in the lowest and highest quartiles of local hazard within each income group. b, Median GCIRI and interquartile range across within-group deciles of the local hazard ratio H, the mean ratio of a city's hazard intensities to the national means of the same hazards (Methods). c, Weakest capacity by city population class, with 3,981, 1,363, 431, 52 and 35 cities from the smallest to the largest class. Strengths are direction-corrected so that higher values are better.</t>
+          <t>a, Mean GCIRI of cities in the weakest (open circles) and strongest (filled circles) quartiles of local hazard within each income group. b, Median GCIRI and interquartile range across within-group deciles of the local hazard ratio H, the mean ratio of a city's hazard intensities to the national means of the same hazards (Methods). c, Mean GCIRI by city population class and income group. Open symbols mark classes with fewer than ten cities, with the number of cities shown. d, Weakest capacity by city population class, with 3,981, 1,363, 431, 52 and 35 cities from the smallest to the largest class. Strengths are direction-corrected so that higher values are better.</t>
         </is>
       </c>
     </row>
@@ -590,13 +590,13 @@
         <v>821</v>
       </c>
       <c r="C2" t="n">
-        <v>87.04504854368932</v>
+        <v>87.16582524271843</v>
       </c>
       <c r="D2" t="n">
-        <v>80.03658536585365</v>
+        <v>80.03043902439023</v>
       </c>
       <c r="E2" t="n">
-        <v>7.008463177835665</v>
+        <v>7.135386218328193</v>
       </c>
     </row>
     <row r="3">
@@ -609,13 +609,13 @@
         <v>1979</v>
       </c>
       <c r="C3" t="n">
-        <v>72.16650505050505</v>
+        <v>72.17535353535354</v>
       </c>
       <c r="D3" t="n">
-        <v>56.6570101010101</v>
+        <v>56.66555555555556</v>
       </c>
       <c r="E3" t="n">
-        <v>15.50949494949495</v>
+        <v>15.50979797979798</v>
       </c>
     </row>
     <row r="4">
@@ -647,13 +647,13 @@
         <v>495</v>
       </c>
       <c r="C5" t="n">
-        <v>39.08451612903225</v>
+        <v>39.08217741935484</v>
       </c>
       <c r="D5" t="n">
         <v>11.49024193548387</v>
       </c>
       <c r="E5" t="n">
-        <v>27.59427419354838</v>
+        <v>27.59193548387097</v>
       </c>
     </row>
   </sheetData>
@@ -720,13 +720,13 @@
         <v>0.6999</v>
       </c>
       <c r="D2" t="n">
-        <v>87.76000000000001</v>
+        <v>87.87</v>
       </c>
       <c r="E2" t="n">
         <v>84.43000000000001</v>
       </c>
       <c r="F2" t="n">
-        <v>92.64</v>
+        <v>92.995</v>
       </c>
       <c r="G2" t="n">
         <v>83</v>
@@ -745,13 +745,13 @@
         <v>0.7479</v>
       </c>
       <c r="D3" t="n">
-        <v>88.90000000000001</v>
+        <v>88.74000000000001</v>
       </c>
       <c r="E3" t="n">
         <v>83.6525</v>
       </c>
       <c r="F3" t="n">
-        <v>92.84999999999999</v>
+        <v>93.07250000000001</v>
       </c>
       <c r="G3" t="n">
         <v>82</v>
@@ -770,13 +770,13 @@
         <v>0.78235</v>
       </c>
       <c r="D4" t="n">
-        <v>88.16</v>
+        <v>88.16999999999999</v>
       </c>
       <c r="E4" t="n">
-        <v>81.60249999999999</v>
+        <v>81.535</v>
       </c>
       <c r="F4" t="n">
-        <v>91.795</v>
+        <v>91.77249999999999</v>
       </c>
       <c r="G4" t="n">
         <v>82</v>
@@ -795,13 +795,13 @@
         <v>0.8228</v>
       </c>
       <c r="D5" t="n">
-        <v>88.44</v>
+        <v>88.405</v>
       </c>
       <c r="E5" t="n">
-        <v>82.5275</v>
+        <v>82.83750000000001</v>
       </c>
       <c r="F5" t="n">
-        <v>92.3275</v>
+        <v>92.4025</v>
       </c>
       <c r="G5" t="n">
         <v>82</v>
@@ -820,13 +820,13 @@
         <v>0.8647499999999999</v>
       </c>
       <c r="D6" t="n">
-        <v>85.215</v>
+        <v>85.30500000000001</v>
       </c>
       <c r="E6" t="n">
         <v>79.9875</v>
       </c>
       <c r="F6" t="n">
-        <v>89.50750000000001</v>
+        <v>89.505</v>
       </c>
       <c r="G6" t="n">
         <v>82</v>
@@ -845,13 +845,13 @@
         <v>0.91095</v>
       </c>
       <c r="D7" t="n">
-        <v>85.13999999999999</v>
+        <v>85.375</v>
       </c>
       <c r="E7" t="n">
         <v>78.7</v>
       </c>
       <c r="F7" t="n">
-        <v>90.39</v>
+        <v>90.38249999999999</v>
       </c>
       <c r="G7" t="n">
         <v>82</v>
@@ -870,13 +870,13 @@
         <v>0.97205</v>
       </c>
       <c r="D8" t="n">
-        <v>85.2</v>
+        <v>85.265</v>
       </c>
       <c r="E8" t="n">
-        <v>75.16250000000001</v>
+        <v>75.2375</v>
       </c>
       <c r="F8" t="n">
-        <v>92.75749999999999</v>
+        <v>93.01000000000001</v>
       </c>
       <c r="G8" t="n">
         <v>82</v>
@@ -895,13 +895,13 @@
         <v>1.0577</v>
       </c>
       <c r="D9" t="n">
-        <v>82.96000000000001</v>
+        <v>83.27500000000001</v>
       </c>
       <c r="E9" t="n">
         <v>73.82000000000001</v>
       </c>
       <c r="F9" t="n">
-        <v>89.77499999999999</v>
+        <v>90.0975</v>
       </c>
       <c r="G9" t="n">
         <v>82</v>
@@ -920,13 +920,13 @@
         <v>1.20375</v>
       </c>
       <c r="D10" t="n">
-        <v>87.09</v>
+        <v>86.93000000000001</v>
       </c>
       <c r="E10" t="n">
-        <v>80.395</v>
+        <v>80.91249999999999</v>
       </c>
       <c r="F10" t="n">
-        <v>90.9375</v>
+        <v>90.9675</v>
       </c>
       <c r="G10" t="n">
         <v>82</v>
@@ -945,10 +945,10 @@
         <v>1.7714</v>
       </c>
       <c r="D11" t="n">
-        <v>77.02500000000001</v>
+        <v>77.89</v>
       </c>
       <c r="E11" t="n">
-        <v>71.3725</v>
+        <v>70.485</v>
       </c>
       <c r="F11" t="n">
         <v>86.94499999999999</v>
@@ -976,7 +976,7 @@
         <v>70.44750000000001</v>
       </c>
       <c r="F12" t="n">
-        <v>78.91</v>
+        <v>79.185</v>
       </c>
       <c r="G12" t="n">
         <v>198</v>
@@ -1755,13 +1755,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>12.58477769404672</v>
+        <v>12.55965837729214</v>
       </c>
       <c r="C2" t="n">
         <v>21.10022607385079</v>
       </c>
       <c r="D2" t="n">
-        <v>66.31499623210249</v>
+        <v>66.34011554885707</v>
       </c>
       <c r="E2" t="n">
         <v>3981</v>
@@ -1774,13 +1774,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>24.57813646368305</v>
+        <v>24.65150403521644</v>
       </c>
       <c r="C3" t="n">
         <v>24.57813646368305</v>
       </c>
       <c r="D3" t="n">
-        <v>50.8437270726339</v>
+        <v>50.77035950110052</v>
       </c>
       <c r="E3" t="n">
         <v>1363</v>
@@ -1894,7 +1894,7 @@
         <v>539</v>
       </c>
       <c r="D2" t="n">
-        <v>83.51339517625232</v>
+        <v>83.58113172541745</v>
       </c>
     </row>
     <row r="3">
@@ -1912,7 +1912,7 @@
         <v>184</v>
       </c>
       <c r="D3" t="n">
-        <v>84.28038043478261</v>
+        <v>84.18983695652175</v>
       </c>
     </row>
     <row r="4">
@@ -1930,7 +1930,7 @@
         <v>83</v>
       </c>
       <c r="D4" t="n">
-        <v>85.88036144578312</v>
+        <v>85.89746987951807</v>
       </c>
     </row>
     <row r="5">
@@ -1948,7 +1948,7 @@
         <v>9</v>
       </c>
       <c r="D5" t="n">
-        <v>84.73888888888888</v>
+        <v>84.42222222222222</v>
       </c>
     </row>
     <row r="6">
@@ -1966,7 +1966,7 @@
         <v>6</v>
       </c>
       <c r="D6" t="n">
-        <v>86.67666666666666</v>
+        <v>86.795</v>
       </c>
     </row>
     <row r="7">
@@ -1984,7 +1984,7 @@
         <v>1294</v>
       </c>
       <c r="D7" t="n">
-        <v>64.97994590417311</v>
+        <v>64.98615919629057</v>
       </c>
     </row>
     <row r="8">
@@ -2002,7 +2002,7 @@
         <v>511</v>
       </c>
       <c r="D8" t="n">
-        <v>65.56101761252447</v>
+        <v>65.56737769080235</v>
       </c>
     </row>
     <row r="9">
@@ -2020,7 +2020,7 @@
         <v>145</v>
       </c>
       <c r="D9" t="n">
-        <v>66.36606896551724</v>
+        <v>66.38620689655173</v>
       </c>
     </row>
     <row r="10">
@@ -2038,7 +2038,7 @@
         <v>15</v>
       </c>
       <c r="D10" t="n">
-        <v>67.91333333333334</v>
+        <v>67.96933333333332</v>
       </c>
     </row>
     <row r="11">
@@ -2056,7 +2056,7 @@
         <v>14</v>
       </c>
       <c r="D11" t="n">
-        <v>70.42928571428571</v>
+        <v>70.46714285714286</v>
       </c>
     </row>
     <row r="12">
@@ -2074,7 +2074,7 @@
         <v>1749</v>
       </c>
       <c r="D12" t="n">
-        <v>37.74899371069183</v>
+        <v>37.74881074899943</v>
       </c>
     </row>
     <row r="13">
@@ -2164,7 +2164,7 @@
         <v>369</v>
       </c>
       <c r="D17" t="n">
-        <v>29.91376693766938</v>
+        <v>29.9129810298103</v>
       </c>
     </row>
     <row r="18">
@@ -2182,7 +2182,7 @@
         <v>90</v>
       </c>
       <c r="D18" t="n">
-        <v>23.21766666666667</v>
+        <v>23.21711111111111</v>
       </c>
     </row>
     <row r="19">

</xml_diff>